<commit_message>
02 junio 2022 v1
</commit_message>
<xml_diff>
--- a/_downloads/20bbe8db6f11f76bcbad1b990f5a24de/Estados Financieros-Supermercado Euro 2019-2020.xlsx
+++ b/_downloads/20bbe8db6f11f76bcbad1b990f5a24de/Estados Financieros-Supermercado Euro 2019-2020.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Talleres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76131E56-9B06-4360-BC9E-0A10EE4D1742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F87F0B-E557-4D47-9BDF-B000B21FE30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{320BED3A-7130-41F8-B37B-3FDC6BE527E6}"/>
   </bookViews>
@@ -231,7 +231,7 @@
     <t>Utilidad neta</t>
   </si>
   <si>
-    <t>Depreciaciones y Amortizaciones año 2020</t>
+    <t>Depreciaciones y Amortizaciones</t>
   </si>
 </sst>
 </file>
@@ -347,12 +347,6 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="6" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -364,6 +358,12 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma 28" xfId="2" xr:uid="{44D01C6C-25D7-407A-A5A1-5A5097C851DB}"/>
@@ -683,23 +683,23 @@
   <dimension ref="A1:C74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.5703125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="47.5703125" style="7" customWidth="1"/>
     <col min="2" max="3" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3"/>
+      <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>2020</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="2">
         <v>2019</v>
       </c>
     </row>
@@ -707,10 +707,10 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>13474829</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>10620685</v>
       </c>
     </row>
@@ -718,10 +718,10 @@
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="3">
         <v>6454100</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="3">
         <v>6301862</v>
       </c>
     </row>
@@ -729,10 +729,10 @@
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>30641796</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>27530459</v>
       </c>
     </row>
@@ -740,10 +740,10 @@
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <v>6334414</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="3">
         <v>6203382</v>
       </c>
     </row>
@@ -751,43 +751,43 @@
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>56905139</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <v>50656388</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="4">
         <f>SUM(B9:B10)</f>
         <v>56905139</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="4">
         <f>SUM(C9:C10)</f>
         <v>50656388</v>
       </c>
@@ -796,10 +796,10 @@
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <v>33010611</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>25660941</v>
       </c>
     </row>
@@ -807,10 +807,10 @@
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>49681443</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <v>46412843</v>
       </c>
     </row>
@@ -818,10 +818,10 @@
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="3">
         <v>3257214</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="3">
         <v>3211841</v>
       </c>
     </row>
@@ -829,38 +829,38 @@
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
     </row>
     <row r="18" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
     </row>
     <row r="19" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="3">
         <v>11743579</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>11609324</v>
       </c>
     </row>
@@ -868,45 +868,45 @@
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
     </row>
     <row r="21" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="6">
+      <c r="B23" s="4">
         <f>SUM(B12:B22)</f>
         <v>97692847</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="4">
         <f t="shared" ref="C23" si="0">SUM(C12:C22)</f>
         <v>86894949</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="6">
+      <c r="B24" s="4">
         <f>+B11+B23</f>
         <v>154597986</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="4">
         <f t="shared" ref="C24" si="1">+C11+C23</f>
         <v>137551337</v>
       </c>
@@ -915,10 +915,10 @@
       <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="3">
         <v>1905658</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="3">
         <v>1731401</v>
       </c>
     </row>
@@ -926,18 +926,18 @@
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="6">
+      <c r="B27" s="4">
         <f>SUM(B25:B26)</f>
         <v>1905658</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="4">
         <f t="shared" ref="C27" si="2">SUM(C25:C26)</f>
         <v>1731401</v>
       </c>
@@ -946,10 +946,10 @@
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28" s="3">
         <v>51802340</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="3">
         <v>50433296</v>
       </c>
     </row>
@@ -957,17 +957,17 @@
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
     </row>
     <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="3">
         <v>4404113</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="3">
         <v>4489396</v>
       </c>
     </row>
@@ -975,10 +975,10 @@
       <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="3">
         <v>731663</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="3">
         <v>632209</v>
       </c>
     </row>
@@ -986,11 +986,11 @@
       <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="6">
+      <c r="B32" s="4">
         <f>SUM(B27:B31)</f>
         <v>58843774</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="4">
         <f>SUM(C27:C31)</f>
         <v>57286302</v>
       </c>
@@ -999,18 +999,18 @@
       <c r="A33" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
     </row>
     <row r="34" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B34" s="4">
         <f>SUM(B32:B33)</f>
         <v>58843774</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="4">
         <f t="shared" ref="C34" si="3">SUM(C32:C33)</f>
         <v>57286302</v>
       </c>
@@ -1019,25 +1019,25 @@
       <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
     </row>
     <row r="36" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
     </row>
     <row r="37" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="4">
         <f>SUM(B35:B36)</f>
         <v>0</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="4">
         <f t="shared" ref="C37" si="4">SUM(C35:C36)</f>
         <v>0</v>
       </c>
@@ -1046,19 +1046,19 @@
       <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="5">
+      <c r="B38" s="3">
         <v>295657</v>
       </c>
-      <c r="C38" s="5"/>
+      <c r="C38" s="3"/>
     </row>
     <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B39" s="3">
         <v>17055268</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="3">
         <v>15937184</v>
       </c>
     </row>
@@ -1066,17 +1066,17 @@
       <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
     </row>
     <row r="41" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B41" s="5">
+      <c r="B41" s="3">
         <v>34264426</v>
       </c>
-      <c r="C41" s="5">
+      <c r="C41" s="3">
         <v>28137179</v>
       </c>
     </row>
@@ -1084,31 +1084,31 @@
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
     </row>
     <row r="43" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
+      <c r="A43" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B43" s="6">
+      <c r="B43" s="4">
         <f>SUM(B37:B42)</f>
         <v>51615351</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C43" s="4">
         <f t="shared" ref="C43" si="5">SUM(C37:C42)</f>
         <v>44074363</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
+      <c r="A44" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B44" s="6">
+      <c r="B44" s="4">
         <f>+B34+B43</f>
         <v>110459125</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C44" s="4">
         <f t="shared" ref="C44" si="6">+C34+C43</f>
         <v>101360665</v>
       </c>
@@ -1117,10 +1117,10 @@
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="5">
+      <c r="B45" s="3">
         <v>2000000</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C45" s="3">
         <v>2000000</v>
       </c>
     </row>
@@ -1128,10 +1128,10 @@
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B46" s="3">
         <v>3795156</v>
       </c>
-      <c r="C46" s="5">
+      <c r="C46" s="3">
         <v>3795156</v>
       </c>
     </row>
@@ -1139,24 +1139,24 @@
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
     </row>
     <row r="48" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
     </row>
     <row r="49" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="5">
+      <c r="B49" s="3">
         <v>13425353</v>
       </c>
-      <c r="C49" s="5">
+      <c r="C49" s="3">
         <v>11093346</v>
       </c>
     </row>
@@ -1164,52 +1164,52 @@
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B50" s="3">
         <v>24918352</v>
       </c>
-      <c r="C50" s="5">
+      <c r="C50" s="3">
         <v>19302170</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
+      <c r="A51" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B51" s="6">
+      <c r="B51" s="4">
         <f>SUM(B45:B50)</f>
         <v>44138861</v>
       </c>
-      <c r="C51" s="6">
+      <c r="C51" s="4">
         <f t="shared" ref="C51" si="7">SUM(C45:C50)</f>
         <v>36190672</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="7" t="s">
+      <c r="A52" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B52" s="6">
+      <c r="B52" s="4">
         <f>+B51+B44</f>
         <v>154597986</v>
       </c>
-      <c r="C52" s="6">
+      <c r="C52" s="4">
         <f t="shared" ref="C52" si="8">+C51+C44</f>
         <v>137551337</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C56" s="3"/>
+      <c r="C56" s="9"/>
     </row>
     <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
-      <c r="B57" s="4">
+      <c r="B57" s="2">
         <v>2020</v>
       </c>
-      <c r="C57" s="4">
+      <c r="C57" s="2">
         <v>2019</v>
       </c>
     </row>
@@ -1217,10 +1217,10 @@
       <c r="A58" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B58" s="5">
+      <c r="B58" s="3">
         <v>414219785</v>
       </c>
-      <c r="C58" s="5">
+      <c r="C58" s="3">
         <v>384684517</v>
       </c>
     </row>
@@ -1228,22 +1228,22 @@
       <c r="A59" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B59" s="3">
         <v>326459104</v>
       </c>
-      <c r="C59" s="5">
+      <c r="C59" s="3">
         <v>306083749</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="7" t="s">
+      <c r="A60" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B60" s="6">
+      <c r="B60" s="4">
         <f>+B58-B59</f>
         <v>87760681</v>
       </c>
-      <c r="C60" s="6">
+      <c r="C60" s="4">
         <f>+C58-C59</f>
         <v>78600768</v>
       </c>
@@ -1252,10 +1252,10 @@
       <c r="A61" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B61" s="5">
+      <c r="B61" s="3">
         <v>7142089</v>
       </c>
-      <c r="C61" s="5">
+      <c r="C61" s="3">
         <v>3735383</v>
       </c>
     </row>
@@ -1263,10 +1263,10 @@
       <c r="A62" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B62" s="5">
+      <c r="B62" s="3">
         <v>73350136</v>
       </c>
-      <c r="C62" s="5">
+      <c r="C62" s="3">
         <v>66675523</v>
       </c>
     </row>
@@ -1274,10 +1274,10 @@
       <c r="A63" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B63" s="5">
+      <c r="B63" s="3">
         <v>4428051</v>
       </c>
-      <c r="C63" s="5">
+      <c r="C63" s="3">
         <v>4443572</v>
       </c>
     </row>
@@ -1285,10 +1285,10 @@
       <c r="A64" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B64" s="3">
         <v>450596</v>
       </c>
-      <c r="C64" s="5">
+      <c r="C64" s="3">
         <v>799715</v>
       </c>
     </row>
@@ -1296,18 +1296,18 @@
       <c r="A65" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
     </row>
     <row r="66" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="7" t="s">
+      <c r="A66" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B66" s="6">
+      <c r="B66" s="4">
         <f>+B60+B61-B62-B63-B64+B65</f>
         <v>16673987</v>
       </c>
-      <c r="C66" s="6">
+      <c r="C66" s="4">
         <f>+C60+C61-C62-C63-C64+C65</f>
         <v>10417341</v>
       </c>
@@ -1316,10 +1316,10 @@
       <c r="A67" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B67" s="5">
+      <c r="B67" s="3">
         <v>331535</v>
       </c>
-      <c r="C67" s="5">
+      <c r="C67" s="3">
         <v>167408</v>
       </c>
     </row>
@@ -1327,22 +1327,22 @@
       <c r="A68" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B68" s="5">
+      <c r="B68" s="3">
         <v>6916845</v>
       </c>
-      <c r="C68" s="5">
+      <c r="C68" s="3">
         <v>6935685</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="7" t="s">
+      <c r="A69" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B69" s="6">
+      <c r="B69" s="4">
         <f>+B66+B67-B68</f>
         <v>10088677</v>
       </c>
-      <c r="C69" s="6">
+      <c r="C69" s="4">
         <f>+C66+C67-C68</f>
         <v>3649064</v>
       </c>
@@ -1351,42 +1351,44 @@
       <c r="A70" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B70" s="3">
         <v>2140488</v>
       </c>
-      <c r="C70" s="5">
+      <c r="C70" s="3">
         <v>1317057</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="7" t="s">
+      <c r="A71" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B71" s="6">
+      <c r="B71" s="4">
         <f>+B69-B70</f>
         <v>7948189</v>
       </c>
-      <c r="C71" s="6">
+      <c r="C71" s="4">
         <f>+C69-C70</f>
         <v>2332007</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B72" s="8"/>
-      <c r="C72" s="8"/>
+      <c r="B72" s="6"/>
+      <c r="C72" s="6"/>
     </row>
     <row r="73" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B73" s="5">
+      <c r="B73" s="3">
+        <v>4435926</v>
+      </c>
+      <c r="C73" s="3">
         <v>5266447</v>
       </c>
-      <c r="C73" s="8"/>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
+      <c r="B74" s="6"/>
+      <c r="C74" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
13 junio 2022 v1
</commit_message>
<xml_diff>
--- a/_downloads/20bbe8db6f11f76bcbad1b990f5a24de/Estados Financieros-Supermercado Euro 2019-2020.xlsx
+++ b/_downloads/20bbe8db6f11f76bcbad1b990f5a24de/Estados Financieros-Supermercado Euro 2019-2020.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Talleres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F87F0B-E557-4D47-9BDF-B000B21FE30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791E983C-941B-47A9-9E69-083AE40E9AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{320BED3A-7130-41F8-B37B-3FDC6BE527E6}"/>
   </bookViews>
@@ -697,10 +697,10 @@
     <row r="2" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2">
+        <v>2019</v>
+      </c>
+      <c r="C2" s="2">
         <v>2020</v>
-      </c>
-      <c r="C2" s="2">
-        <v>2019</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -708,10 +708,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
+        <v>10620685</v>
+      </c>
+      <c r="C3" s="3">
         <v>13474829</v>
-      </c>
-      <c r="C3" s="3">
-        <v>10620685</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -719,10 +719,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3">
+        <v>6301862</v>
+      </c>
+      <c r="C4" s="3">
         <v>6454100</v>
-      </c>
-      <c r="C4" s="3">
-        <v>6301862</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -730,10 +730,10 @@
         <v>5</v>
       </c>
       <c r="B5" s="3">
+        <v>27530459</v>
+      </c>
+      <c r="C5" s="3">
         <v>30641796</v>
-      </c>
-      <c r="C5" s="3">
-        <v>27530459</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -741,10 +741,10 @@
         <v>7</v>
       </c>
       <c r="B6" s="3">
+        <v>6203382</v>
+      </c>
+      <c r="C6" s="3">
         <v>6334414</v>
-      </c>
-      <c r="C6" s="3">
-        <v>6203382</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -773,10 +773,10 @@
         <v>11</v>
       </c>
       <c r="B10" s="3">
+        <v>50656388</v>
+      </c>
+      <c r="C10" s="3">
         <v>56905139</v>
-      </c>
-      <c r="C10" s="3">
-        <v>50656388</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -785,11 +785,11 @@
       </c>
       <c r="B11" s="4">
         <f>SUM(B9:B10)</f>
-        <v>56905139</v>
+        <v>50656388</v>
       </c>
       <c r="C11" s="4">
         <f>SUM(C9:C10)</f>
-        <v>50656388</v>
+        <v>56905139</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -797,10 +797,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="3">
+        <v>25660941</v>
+      </c>
+      <c r="C12" s="3">
         <v>33010611</v>
-      </c>
-      <c r="C12" s="3">
-        <v>25660941</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -808,10 +808,10 @@
         <v>2</v>
       </c>
       <c r="B13" s="3">
+        <v>46412843</v>
+      </c>
+      <c r="C13" s="3">
         <v>49681443</v>
-      </c>
-      <c r="C13" s="3">
-        <v>46412843</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -819,10 +819,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3">
+        <v>3211841</v>
+      </c>
+      <c r="C14" s="3">
         <v>3257214</v>
-      </c>
-      <c r="C14" s="3">
-        <v>3211841</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -858,10 +858,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="3">
+        <v>11609324</v>
+      </c>
+      <c r="C19" s="3">
         <v>11743579</v>
-      </c>
-      <c r="C19" s="3">
-        <v>11609324</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -890,12 +890,12 @@
         <v>22</v>
       </c>
       <c r="B23" s="4">
-        <f>SUM(B12:B22)</f>
+        <f t="shared" ref="B23" si="0">SUM(B12:B22)</f>
+        <v>86894949</v>
+      </c>
+      <c r="C23" s="4">
+        <f>SUM(C12:C22)</f>
         <v>97692847</v>
-      </c>
-      <c r="C23" s="4">
-        <f t="shared" ref="C23" si="0">SUM(C12:C22)</f>
-        <v>86894949</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -903,12 +903,12 @@
         <v>23</v>
       </c>
       <c r="B24" s="4">
-        <f>+B11+B23</f>
+        <f t="shared" ref="B24" si="1">+B11+B23</f>
+        <v>137551337</v>
+      </c>
+      <c r="C24" s="4">
+        <f>+C11+C23</f>
         <v>154597986</v>
-      </c>
-      <c r="C24" s="4">
-        <f t="shared" ref="C24" si="1">+C11+C23</f>
-        <v>137551337</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -916,10 +916,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3">
+        <v>1731401</v>
+      </c>
+      <c r="C25" s="3">
         <v>1905658</v>
-      </c>
-      <c r="C25" s="3">
-        <v>1731401</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -934,12 +934,12 @@
         <v>26</v>
       </c>
       <c r="B27" s="4">
-        <f>SUM(B25:B26)</f>
+        <f t="shared" ref="B27" si="2">SUM(B25:B26)</f>
+        <v>1731401</v>
+      </c>
+      <c r="C27" s="4">
+        <f>SUM(C25:C26)</f>
         <v>1905658</v>
-      </c>
-      <c r="C27" s="4">
-        <f t="shared" ref="C27" si="2">SUM(C25:C26)</f>
-        <v>1731401</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -947,10 +947,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3">
+        <v>50433296</v>
+      </c>
+      <c r="C28" s="3">
         <v>51802340</v>
-      </c>
-      <c r="C28" s="3">
-        <v>50433296</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -965,10 +965,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3">
+        <v>4489396</v>
+      </c>
+      <c r="C30" s="3">
         <v>4404113</v>
-      </c>
-      <c r="C30" s="3">
-        <v>4489396</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -976,10 +976,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3">
+        <v>632209</v>
+      </c>
+      <c r="C31" s="3">
         <v>731663</v>
-      </c>
-      <c r="C31" s="3">
-        <v>632209</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -988,11 +988,11 @@
       </c>
       <c r="B32" s="4">
         <f>SUM(B27:B31)</f>
-        <v>58843774</v>
+        <v>57286302</v>
       </c>
       <c r="C32" s="4">
         <f>SUM(C27:C31)</f>
-        <v>57286302</v>
+        <v>58843774</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1007,12 +1007,12 @@
         <v>33</v>
       </c>
       <c r="B34" s="4">
-        <f>SUM(B32:B33)</f>
+        <f t="shared" ref="B34" si="3">SUM(B32:B33)</f>
+        <v>57286302</v>
+      </c>
+      <c r="C34" s="4">
+        <f>SUM(C32:C33)</f>
         <v>58843774</v>
-      </c>
-      <c r="C34" s="4">
-        <f t="shared" ref="C34" si="3">SUM(C32:C33)</f>
-        <v>57286302</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1034,11 +1034,11 @@
         <v>36</v>
       </c>
       <c r="B37" s="4">
-        <f>SUM(B35:B36)</f>
+        <f t="shared" ref="B37" si="4">SUM(B35:B36)</f>
         <v>0</v>
       </c>
       <c r="C37" s="4">
-        <f t="shared" ref="C37" si="4">SUM(C35:C36)</f>
+        <f>SUM(C35:C36)</f>
         <v>0</v>
       </c>
     </row>
@@ -1046,20 +1046,20 @@
       <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="3">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3">
         <v>295657</v>
       </c>
-      <c r="C38" s="3"/>
     </row>
     <row r="39" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="3">
+        <v>15937184</v>
+      </c>
+      <c r="C39" s="3">
         <v>17055268</v>
-      </c>
-      <c r="C39" s="3">
-        <v>15937184</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1074,10 +1074,10 @@
         <v>4</v>
       </c>
       <c r="B41" s="3">
+        <v>28137179</v>
+      </c>
+      <c r="C41" s="3">
         <v>34264426</v>
-      </c>
-      <c r="C41" s="3">
-        <v>28137179</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1092,12 +1092,12 @@
         <v>41</v>
       </c>
       <c r="B43" s="4">
-        <f>SUM(B37:B42)</f>
+        <f t="shared" ref="B43" si="5">SUM(B37:B42)</f>
+        <v>44074363</v>
+      </c>
+      <c r="C43" s="4">
+        <f>SUM(C37:C42)</f>
         <v>51615351</v>
-      </c>
-      <c r="C43" s="4">
-        <f t="shared" ref="C43" si="5">SUM(C37:C42)</f>
-        <v>44074363</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1105,12 +1105,12 @@
         <v>42</v>
       </c>
       <c r="B44" s="4">
-        <f>+B34+B43</f>
+        <f t="shared" ref="B44" si="6">+B34+B43</f>
+        <v>101360665</v>
+      </c>
+      <c r="C44" s="4">
+        <f>+C34+C43</f>
         <v>110459125</v>
-      </c>
-      <c r="C44" s="4">
-        <f t="shared" ref="C44" si="6">+C34+C43</f>
-        <v>101360665</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1154,10 +1154,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="3">
+        <v>11093346</v>
+      </c>
+      <c r="C49" s="3">
         <v>13425353</v>
-      </c>
-      <c r="C49" s="3">
-        <v>11093346</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1165,10 +1165,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="3">
+        <v>19302170</v>
+      </c>
+      <c r="C50" s="3">
         <v>24918352</v>
-      </c>
-      <c r="C50" s="3">
-        <v>19302170</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1176,12 +1176,12 @@
         <v>49</v>
       </c>
       <c r="B51" s="4">
-        <f>SUM(B45:B50)</f>
+        <f t="shared" ref="B51" si="7">SUM(B45:B50)</f>
+        <v>36190672</v>
+      </c>
+      <c r="C51" s="4">
+        <f>SUM(C45:C50)</f>
         <v>44138861</v>
-      </c>
-      <c r="C51" s="4">
-        <f t="shared" ref="C51" si="7">SUM(C45:C50)</f>
-        <v>36190672</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1189,12 +1189,12 @@
         <v>50</v>
       </c>
       <c r="B52" s="4">
-        <f>+B51+B44</f>
+        <f t="shared" ref="B52" si="8">+B51+B44</f>
+        <v>137551337</v>
+      </c>
+      <c r="C52" s="4">
+        <f>+C51+C44</f>
         <v>154597986</v>
-      </c>
-      <c r="C52" s="4">
-        <f t="shared" ref="C52" si="8">+C51+C44</f>
-        <v>137551337</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1207,10 +1207,10 @@
     <row r="57" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="2">
+        <v>2019</v>
+      </c>
+      <c r="C57" s="2">
         <v>2020</v>
-      </c>
-      <c r="C57" s="2">
-        <v>2019</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1218,10 +1218,10 @@
         <v>51</v>
       </c>
       <c r="B58" s="3">
+        <v>384684517</v>
+      </c>
+      <c r="C58" s="3">
         <v>414219785</v>
-      </c>
-      <c r="C58" s="3">
-        <v>384684517</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1229,10 +1229,10 @@
         <v>52</v>
       </c>
       <c r="B59" s="3">
+        <v>306083749</v>
+      </c>
+      <c r="C59" s="3">
         <v>326459104</v>
-      </c>
-      <c r="C59" s="3">
-        <v>306083749</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1241,11 +1241,11 @@
       </c>
       <c r="B60" s="4">
         <f>+B58-B59</f>
-        <v>87760681</v>
+        <v>78600768</v>
       </c>
       <c r="C60" s="4">
         <f>+C58-C59</f>
-        <v>78600768</v>
+        <v>87760681</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1253,10 +1253,10 @@
         <v>54</v>
       </c>
       <c r="B61" s="3">
+        <v>3735383</v>
+      </c>
+      <c r="C61" s="3">
         <v>7142089</v>
-      </c>
-      <c r="C61" s="3">
-        <v>3735383</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1264,10 +1264,10 @@
         <v>55</v>
       </c>
       <c r="B62" s="3">
+        <v>66675523</v>
+      </c>
+      <c r="C62" s="3">
         <v>73350136</v>
-      </c>
-      <c r="C62" s="3">
-        <v>66675523</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1275,10 +1275,10 @@
         <v>56</v>
       </c>
       <c r="B63" s="3">
+        <v>4443572</v>
+      </c>
+      <c r="C63" s="3">
         <v>4428051</v>
-      </c>
-      <c r="C63" s="3">
-        <v>4443572</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1286,10 +1286,10 @@
         <v>57</v>
       </c>
       <c r="B64" s="3">
+        <v>799715</v>
+      </c>
+      <c r="C64" s="3">
         <v>450596</v>
-      </c>
-      <c r="C64" s="3">
-        <v>799715</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1305,11 +1305,11 @@
       </c>
       <c r="B66" s="4">
         <f>+B60+B61-B62-B63-B64+B65</f>
-        <v>16673987</v>
+        <v>10417341</v>
       </c>
       <c r="C66" s="4">
         <f>+C60+C61-C62-C63-C64+C65</f>
-        <v>10417341</v>
+        <v>16673987</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1317,10 +1317,10 @@
         <v>60</v>
       </c>
       <c r="B67" s="3">
+        <v>167408</v>
+      </c>
+      <c r="C67" s="3">
         <v>331535</v>
-      </c>
-      <c r="C67" s="3">
-        <v>167408</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1328,10 +1328,10 @@
         <v>61</v>
       </c>
       <c r="B68" s="3">
+        <v>6935685</v>
+      </c>
+      <c r="C68" s="3">
         <v>6916845</v>
-      </c>
-      <c r="C68" s="3">
-        <v>6935685</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1340,11 +1340,11 @@
       </c>
       <c r="B69" s="4">
         <f>+B66+B67-B68</f>
-        <v>10088677</v>
+        <v>3649064</v>
       </c>
       <c r="C69" s="4">
         <f>+C66+C67-C68</f>
-        <v>3649064</v>
+        <v>10088677</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1352,10 +1352,10 @@
         <v>63</v>
       </c>
       <c r="B70" s="3">
+        <v>1317057</v>
+      </c>
+      <c r="C70" s="3">
         <v>2140488</v>
-      </c>
-      <c r="C70" s="3">
-        <v>1317057</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -1364,11 +1364,11 @@
       </c>
       <c r="B71" s="4">
         <f>+B69-B70</f>
-        <v>7948189</v>
+        <v>2332007</v>
       </c>
       <c r="C71" s="4">
         <f>+C69-C70</f>
-        <v>2332007</v>
+        <v>7948189</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1380,10 +1380,10 @@
         <v>65</v>
       </c>
       <c r="B73" s="3">
+        <v>5266447</v>
+      </c>
+      <c r="C73" s="3">
         <v>4435926</v>
-      </c>
-      <c r="C73" s="3">
-        <v>5266447</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>